<commit_message>
added currency year to the cleaned capex_capacity
</commit_message>
<xml_diff>
--- a/clean_data/capex_capacity.xlsx
+++ b/clean_data/capex_capacity.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://iowa-my.sharepoint.com/personal/jjohnson316_uiowa_edu/Documents/Research/codes/clean_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="8" documentId="11_755510A5D32056557D43CAF0505ED87656CD3458" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CB40C31B-8341-47C8-AA7F-81AFD85CD8F8}"/>
+  <xr:revisionPtr revIDLastSave="9" documentId="11_755510A5D32056557D43CAF0505ED87656CD3458" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A78B0D34-1C39-4E42-BEE7-07BEFC05FC57}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -440,7 +440,7 @@
     <col min="3" max="3" width="20.7109375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="17.28515625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="22.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
modified the code to make the plots better
</commit_message>
<xml_diff>
--- a/clean_data/capex_capacity.xlsx
+++ b/clean_data/capex_capacity.xlsx
@@ -973,7 +973,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Membrane technology</t>
+          <t xml:space="preserve">Membrane separation </t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -1005,7 +1005,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Membrane technology</t>
+          <t xml:space="preserve">Membrane separation </t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1037,7 +1037,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Membrane technology</t>
+          <t xml:space="preserve">Membrane separation </t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -1069,7 +1069,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Membrane technology</t>
+          <t xml:space="preserve">Membrane separation </t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1101,7 +1101,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Membrane technology</t>
+          <t xml:space="preserve">Membrane separation </t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -1133,7 +1133,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Membrane technology</t>
+          <t xml:space="preserve">Membrane separation </t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1165,7 +1165,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Membrane technology</t>
+          <t xml:space="preserve">Membrane separation </t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -1197,7 +1197,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Membrane technology</t>
+          <t xml:space="preserve">Membrane separation </t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1229,7 +1229,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Chemical absorption (amine scrubbing)</t>
+          <t>Amine scrubbing</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -1261,7 +1261,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Chemical absorption (amine scrubbing)</t>
+          <t>Amine scrubbing</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1293,7 +1293,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Chemical absorption (amine scrubbing)</t>
+          <t>Amine scrubbing</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -1325,7 +1325,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Chemical absorption (amine scrubbing)</t>
+          <t>Amine scrubbing</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1357,7 +1357,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Chemical absorption (amine scrubbing)</t>
+          <t>Amine scrubbing</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -1389,7 +1389,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Chemical absorption (amine scrubbing)</t>
+          <t>Amine scrubbing</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1421,7 +1421,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Chemical absorption (amine scrubbing)</t>
+          <t>Amine scrubbing</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -1773,7 +1773,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Water scrubbing (high pressure, batchwise, small scale)</t>
+          <t>Water scrubbing</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -1805,7 +1805,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Water scrubbing (rotary coil, Biosling, small scale)</t>
+          <t>Water scrubbing</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -1837,7 +1837,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Water scrubbing (rotary coil, Biosling, small scale)</t>
+          <t>Water scrubbing</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -1869,7 +1869,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Membrane technology</t>
+          <t xml:space="preserve">Membrane separation </t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -1901,7 +1901,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Membrane technology</t>
+          <t xml:space="preserve">Membrane separation </t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -1933,7 +1933,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Membrane technology</t>
+          <t xml:space="preserve">Membrane separation </t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -1965,7 +1965,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Membrane technology</t>
+          <t xml:space="preserve">Membrane separation </t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -1997,7 +1997,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Membrane technology</t>
+          <t xml:space="preserve">Membrane separation </t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -2029,7 +2029,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Membrane technology</t>
+          <t xml:space="preserve">Membrane separation </t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2093,7 +2093,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Water scrubbing with regeneration</t>
+          <t>Water scrubbing</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -2125,7 +2125,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Water scrubbing with regeneration</t>
+          <t>Water scrubbing</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -2477,7 +2477,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Chemical absorption (amine scrubbing)</t>
+          <t>Amine scrubbing</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -2541,7 +2541,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Chemical absorption (amine scrubbing)</t>
+          <t>Amine scrubbing</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -2573,7 +2573,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Chemical absorption (amine scrubbing)</t>
+          <t>Amine scrubbing</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -2605,7 +2605,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Chemical absorption (amine scrubbing)</t>
+          <t>Amine scrubbing</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -2797,7 +2797,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Water scrubbing + PSA (O2/N2 removal)</t>
+          <t>Water scrubbing</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -2829,7 +2829,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Water scrubbing + PSA (O2/N2 removal)</t>
+          <t>Water scrubbing</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -3117,7 +3117,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Chemical absorption (amine scrubbing)</t>
+          <t>Amine scrubbing</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -3149,7 +3149,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Chemical absorption (amine scrubbing)</t>
+          <t>Amine scrubbing</t>
         </is>
       </c>
       <c r="B86" t="n">
@@ -3245,7 +3245,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Membrane technology</t>
+          <t xml:space="preserve">Membrane separation </t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -3277,7 +3277,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Membrane technology</t>
+          <t xml:space="preserve">Membrane separation </t>
         </is>
       </c>
       <c r="B90" t="n">
@@ -3309,7 +3309,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Membrane technology</t>
+          <t xml:space="preserve">Membrane separation </t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -3565,7 +3565,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Chemical absorption (amine scrubbing)</t>
+          <t>Amine scrubbing</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -3597,7 +3597,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Chemical absorption (amine scrubbing)</t>
+          <t>Amine scrubbing</t>
         </is>
       </c>
       <c r="B100" t="n">
@@ -3693,7 +3693,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Membrane technology</t>
+          <t xml:space="preserve">Membrane separation </t>
         </is>
       </c>
       <c r="B103" t="n">
@@ -3725,7 +3725,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Membrane technology</t>
+          <t xml:space="preserve">Membrane separation </t>
         </is>
       </c>
       <c r="B104" t="n">
@@ -3757,7 +3757,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Membrane technology</t>
+          <t xml:space="preserve">Membrane separation </t>
         </is>
       </c>
       <c r="B105" t="n">
@@ -3789,7 +3789,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Siloxane removal system, siloxane-only (ancillary, not upgrading)</t>
+          <t>Siloxane removal system</t>
         </is>
       </c>
       <c r="B106" t="n">

</xml_diff>

<commit_message>
Add levelized cost calculation saved
</commit_message>
<xml_diff>
--- a/clean_data/capex_capacity.xlsx
+++ b/clean_data/capex_capacity.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H106"/>
+  <dimension ref="A1:L106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -444,17 +444,37 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>currency_year</t>
+          <t>source</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
+          <t>year</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>capacity_m3_per_hr</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
           <t>reported_capex_usd</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>reported_capex_usd_2025</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>main_technology</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>main_technology_capex_usd_2025</t>
         </is>
       </c>
     </row>
@@ -480,13 +500,29 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F2" t="n">
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Bauer et al. 2013</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
         <v>2013</v>
       </c>
-      <c r="G2" t="n">
+      <c r="H2" t="n">
+        <v>130</v>
+      </c>
+      <c r="I2" t="n">
         <v>878113.1580000001</v>
       </c>
-      <c r="H2" t="n">
+      <c r="J2" t="n">
+        <v>1258118.05891486</v>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Water scrubbing</t>
+        </is>
+      </c>
+      <c r="L2" t="n">
         <v>1258118.05891486</v>
       </c>
     </row>
@@ -512,13 +548,29 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F3" t="n">
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Bauer et al. 2013</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
         <v>2013</v>
       </c>
-      <c r="G3" t="n">
+      <c r="H3" t="n">
+        <v>250</v>
+      </c>
+      <c r="I3" t="n">
         <v>1342045.05</v>
       </c>
-      <c r="H3" t="n">
+      <c r="J3" t="n">
+        <v>1922817.233632998</v>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Water scrubbing</t>
+        </is>
+      </c>
+      <c r="L3" t="n">
         <v>1922817.233632998</v>
       </c>
     </row>
@@ -544,13 +596,29 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F4" t="n">
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Bauer et al. 2013</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
         <v>2013</v>
       </c>
-      <c r="G4" t="n">
+      <c r="H4" t="n">
+        <v>500</v>
+      </c>
+      <c r="I4" t="n">
         <v>1723209.75</v>
       </c>
-      <c r="H4" t="n">
+      <c r="J4" t="n">
+        <v>2468931.579058699</v>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Water scrubbing</t>
+        </is>
+      </c>
+      <c r="L4" t="n">
         <v>2468931.579058699</v>
       </c>
     </row>
@@ -576,13 +644,29 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F5" t="n">
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Bauer et al. 2013</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
         <v>2013</v>
       </c>
-      <c r="G5" t="n">
+      <c r="H5" t="n">
+        <v>750</v>
+      </c>
+      <c r="I5" t="n">
         <v>1922424.75</v>
       </c>
-      <c r="H5" t="n">
+      <c r="J5" t="n">
+        <v>2754357.195134849</v>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Water scrubbing</t>
+        </is>
+      </c>
+      <c r="L5" t="n">
         <v>2754357.195134849</v>
       </c>
     </row>
@@ -608,13 +692,29 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F6" t="n">
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Bauer et al. 2013</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
         <v>2013</v>
       </c>
-      <c r="G6" t="n">
+      <c r="H6" t="n">
+        <v>1000</v>
+      </c>
+      <c r="I6" t="n">
         <v>2249801.4</v>
       </c>
-      <c r="H6" t="n">
+      <c r="J6" t="n">
+        <v>3223406.624219989</v>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Water scrubbing</t>
+        </is>
+      </c>
+      <c r="L6" t="n">
         <v>3223406.624219989</v>
       </c>
     </row>
@@ -640,13 +740,29 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F7" t="n">
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Bauer et al. 2013</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
         <v>2013</v>
       </c>
-      <c r="G7" t="n">
+      <c r="H7" t="n">
+        <v>1250</v>
+      </c>
+      <c r="I7" t="n">
         <v>2699363.25</v>
       </c>
-      <c r="H7" t="n">
+      <c r="J7" t="n">
+        <v>3867517.097831835</v>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Water scrubbing</t>
+        </is>
+      </c>
+      <c r="L7" t="n">
         <v>3867517.097831835</v>
       </c>
     </row>
@@ -672,13 +788,29 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F8" t="n">
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Bauer et al. 2013</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
         <v>2013</v>
       </c>
-      <c r="G8" t="n">
+      <c r="H8" t="n">
+        <v>1500</v>
+      </c>
+      <c r="I8" t="n">
         <v>3147597</v>
       </c>
-      <c r="H8" t="n">
+      <c r="J8" t="n">
+        <v>4509724.734003173</v>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Water scrubbing</t>
+        </is>
+      </c>
+      <c r="L8" t="n">
         <v>4509724.734003173</v>
       </c>
     </row>
@@ -704,13 +836,29 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F9" t="n">
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Bauer et al. 2013</t>
+        </is>
+      </c>
+      <c r="G9" t="n">
         <v>2013</v>
       </c>
-      <c r="G9" t="n">
+      <c r="H9" t="n">
+        <v>1750</v>
+      </c>
+      <c r="I9" t="n">
         <v>3488586.675</v>
       </c>
-      <c r="H9" t="n">
+      <c r="J9" t="n">
+        <v>4998278.246853516</v>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Water scrubbing</t>
+        </is>
+      </c>
+      <c r="L9" t="n">
         <v>4998278.246853516</v>
       </c>
     </row>
@@ -736,13 +884,29 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F10" t="n">
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Bauer et al. 2013</t>
+        </is>
+      </c>
+      <c r="G10" t="n">
         <v>2013</v>
       </c>
-      <c r="G10" t="n">
+      <c r="H10" t="n">
+        <v>2000</v>
+      </c>
+      <c r="I10" t="n">
         <v>3787741.2</v>
       </c>
-      <c r="H10" t="n">
+      <c r="J10" t="n">
+        <v>5426892.380327869</v>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Water scrubbing</t>
+        </is>
+      </c>
+      <c r="L10" t="n">
         <v>5426892.380327869</v>
       </c>
     </row>
@@ -768,13 +932,29 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F11" t="n">
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Bauer et al. 2013</t>
+        </is>
+      </c>
+      <c r="G11" t="n">
         <v>2013</v>
       </c>
-      <c r="G11" t="n">
+      <c r="H11" t="n">
+        <v>500</v>
+      </c>
+      <c r="I11" t="n">
         <v>1871956.95</v>
       </c>
-      <c r="H11" t="n">
+      <c r="J11" t="n">
+        <v>2682049.372395558</v>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Pressure swing adsorption</t>
+        </is>
+      </c>
+      <c r="L11" t="n">
         <v>2682049.372395558</v>
       </c>
     </row>
@@ -800,13 +980,29 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F12" t="n">
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Bauer et al. 2013</t>
+        </is>
+      </c>
+      <c r="G12" t="n">
         <v>2013</v>
       </c>
-      <c r="G12" t="n">
+      <c r="H12" t="n">
+        <v>750</v>
+      </c>
+      <c r="I12" t="n">
         <v>2323842.975</v>
       </c>
-      <c r="H12" t="n">
+      <c r="J12" t="n">
+        <v>3329489.811528292</v>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Pressure swing adsorption</t>
+        </is>
+      </c>
+      <c r="L12" t="n">
         <v>3329489.811528292</v>
       </c>
     </row>
@@ -832,13 +1028,29 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F13" t="n">
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Bauer et al. 2013</t>
+        </is>
+      </c>
+      <c r="G13" t="n">
         <v>2013</v>
       </c>
-      <c r="G13" t="n">
+      <c r="H13" t="n">
+        <v>1000</v>
+      </c>
+      <c r="I13" t="n">
         <v>2705339.7</v>
       </c>
-      <c r="H13" t="n">
+      <c r="J13" t="n">
+        <v>3876079.86631412</v>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>Pressure swing adsorption</t>
+        </is>
+      </c>
+      <c r="L13" t="n">
         <v>3876079.86631412</v>
       </c>
     </row>
@@ -864,13 +1076,29 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F14" t="n">
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Bauer et al. 2013</t>
+        </is>
+      </c>
+      <c r="G14" t="n">
         <v>2013</v>
       </c>
-      <c r="G14" t="n">
+      <c r="H14" t="n">
+        <v>1250</v>
+      </c>
+      <c r="I14" t="n">
         <v>3043009.125</v>
       </c>
-      <c r="H14" t="n">
+      <c r="J14" t="n">
+        <v>4359876.285563194</v>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>Pressure swing adsorption</t>
+        </is>
+      </c>
+      <c r="L14" t="n">
         <v>4359876.285563194</v>
       </c>
     </row>
@@ -896,13 +1124,29 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F15" t="n">
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Bauer et al. 2013</t>
+        </is>
+      </c>
+      <c r="G15" t="n">
         <v>2013</v>
       </c>
-      <c r="G15" t="n">
+      <c r="H15" t="n">
+        <v>1500</v>
+      </c>
+      <c r="I15" t="n">
         <v>3354780.6</v>
       </c>
-      <c r="H15" t="n">
+      <c r="J15" t="n">
+        <v>4806567.374722369</v>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>Pressure swing adsorption</t>
+        </is>
+      </c>
+      <c r="L15" t="n">
         <v>4806567.374722369</v>
       </c>
     </row>
@@ -928,13 +1172,29 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F16" t="n">
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Bauer et al. 2013</t>
+        </is>
+      </c>
+      <c r="G16" t="n">
         <v>2013</v>
       </c>
-      <c r="G16" t="n">
+      <c r="H16" t="n">
+        <v>1750</v>
+      </c>
+      <c r="I16" t="n">
         <v>3639658.05</v>
       </c>
-      <c r="H16" t="n">
+      <c r="J16" t="n">
+        <v>5214726.005711264</v>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>Pressure swing adsorption</t>
+        </is>
+      </c>
+      <c r="L16" t="n">
         <v>5214726.005711264</v>
       </c>
     </row>
@@ -960,20 +1220,36 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F17" t="n">
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Bauer et al. 2013</t>
+        </is>
+      </c>
+      <c r="G17" t="n">
         <v>2013</v>
       </c>
-      <c r="G17" t="n">
+      <c r="H17" t="n">
+        <v>2000</v>
+      </c>
+      <c r="I17" t="n">
         <v>3907270.2</v>
       </c>
-      <c r="H17" t="n">
+      <c r="J17" t="n">
+        <v>5598147.749973559</v>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>Pressure swing adsorption</t>
+        </is>
+      </c>
+      <c r="L17" t="n">
         <v>5598147.749973559</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Membrane separation </t>
+          <t>Membrane separation</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -992,20 +1268,36 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F18" t="n">
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Bauer et al. 2013</t>
+        </is>
+      </c>
+      <c r="G18" t="n">
         <v>2013</v>
       </c>
-      <c r="G18" t="n">
+      <c r="H18" t="n">
+        <v>140</v>
+      </c>
+      <c r="I18" t="n">
         <v>920187.366</v>
       </c>
-      <c r="H18" t="n">
+      <c r="J18" t="n">
+        <v>1318399.949030143</v>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>Membrane separation</t>
+        </is>
+      </c>
+      <c r="L18" t="n">
         <v>1318399.949030143</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Membrane separation </t>
+          <t>Membrane separation</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1024,20 +1316,36 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F19" t="n">
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Bauer et al. 2013</t>
+        </is>
+      </c>
+      <c r="G19" t="n">
         <v>2013</v>
       </c>
-      <c r="G19" t="n">
+      <c r="H19" t="n">
+        <v>200</v>
+      </c>
+      <c r="I19" t="n">
         <v>1025558.82</v>
       </c>
-      <c r="H19" t="n">
+      <c r="J19" t="n">
+        <v>1469371.071560021</v>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>Membrane separation</t>
+        </is>
+      </c>
+      <c r="L19" t="n">
         <v>1469371.071560021</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Membrane separation </t>
+          <t>Membrane separation</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -1056,20 +1364,36 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F20" t="n">
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Bauer et al. 2013</t>
+        </is>
+      </c>
+      <c r="G20" t="n">
         <v>2013</v>
       </c>
-      <c r="G20" t="n">
+      <c r="H20" t="n">
+        <v>400</v>
+      </c>
+      <c r="I20" t="n">
         <v>1446035.28</v>
       </c>
-      <c r="H20" t="n">
+      <c r="J20" t="n">
+        <v>2071809.405224749</v>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>Membrane separation</t>
+        </is>
+      </c>
+      <c r="L20" t="n">
         <v>2071809.405224749</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Membrane separation </t>
+          <t>Membrane separation</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1088,20 +1412,36 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F21" t="n">
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Bauer et al. 2013</t>
+        </is>
+      </c>
+      <c r="G21" t="n">
         <v>2013</v>
       </c>
-      <c r="G21" t="n">
+      <c r="H21" t="n">
+        <v>600</v>
+      </c>
+      <c r="I21" t="n">
         <v>1906089.12</v>
       </c>
-      <c r="H21" t="n">
+      <c r="J21" t="n">
+        <v>2730952.294616605</v>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>Membrane separation</t>
+        </is>
+      </c>
+      <c r="L21" t="n">
         <v>2730952.294616605</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Membrane separation </t>
+          <t>Membrane separation</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -1120,20 +1460,36 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F22" t="n">
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Bauer et al. 2013</t>
+        </is>
+      </c>
+      <c r="G22" t="n">
         <v>2013</v>
       </c>
-      <c r="G22" t="n">
+      <c r="H22" t="n">
+        <v>800</v>
+      </c>
+      <c r="I22" t="n">
         <v>2203583.52</v>
       </c>
-      <c r="H22" t="n">
+      <c r="J22" t="n">
+        <v>3157187.881290323</v>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>Membrane separation</t>
+        </is>
+      </c>
+      <c r="L22" t="n">
         <v>3157187.881290323</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t xml:space="preserve">Membrane separation </t>
+          <t>Membrane separation</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1152,20 +1508,36 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F23" t="n">
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Bauer et al. 2013</t>
+        </is>
+      </c>
+      <c r="G23" t="n">
         <v>2013</v>
       </c>
-      <c r="G23" t="n">
+      <c r="H23" t="n">
+        <v>1000</v>
+      </c>
+      <c r="I23" t="n">
         <v>2580498.3</v>
       </c>
-      <c r="H23" t="n">
+      <c r="J23" t="n">
+        <v>3697213.146906399</v>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>Membrane separation</t>
+        </is>
+      </c>
+      <c r="L23" t="n">
         <v>3697213.146906399</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve">Membrane separation </t>
+          <t>Membrane separation</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -1184,20 +1556,36 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F24" t="n">
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Bauer et al. 2013</t>
+        </is>
+      </c>
+      <c r="G24" t="n">
         <v>2013</v>
       </c>
-      <c r="G24" t="n">
+      <c r="H24" t="n">
+        <v>1200</v>
+      </c>
+      <c r="I24" t="n">
         <v>3055161.24</v>
       </c>
-      <c r="H24" t="n">
+      <c r="J24" t="n">
+        <v>4377287.24814384</v>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>Membrane separation</t>
+        </is>
+      </c>
+      <c r="L24" t="n">
         <v>4377287.24814384</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Membrane separation </t>
+          <t>Membrane separation</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1216,13 +1604,29 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F25" t="n">
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Bauer et al. 2013</t>
+        </is>
+      </c>
+      <c r="G25" t="n">
         <v>2013</v>
       </c>
-      <c r="G25" t="n">
+      <c r="H25" t="n">
+        <v>1400</v>
+      </c>
+      <c r="I25" t="n">
         <v>3400732.86</v>
       </c>
-      <c r="H25" t="n">
+      <c r="J25" t="n">
+        <v>4872405.550163935</v>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>Membrane separation</t>
+        </is>
+      </c>
+      <c r="L25" t="n">
         <v>4872405.550163935</v>
       </c>
     </row>
@@ -1248,13 +1652,29 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F26" t="n">
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Bauer et al. 2013</t>
+        </is>
+      </c>
+      <c r="G26" t="n">
         <v>2013</v>
       </c>
-      <c r="G26" t="n">
+      <c r="H26" t="n">
+        <v>600</v>
+      </c>
+      <c r="I26" t="n">
         <v>2542780.26</v>
       </c>
-      <c r="H26" t="n">
+      <c r="J26" t="n">
+        <v>3643172.563595981</v>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>Amine scrubbing</t>
+        </is>
+      </c>
+      <c r="L26" t="n">
         <v>3643172.563595981</v>
       </c>
     </row>
@@ -1280,13 +1700,29 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F27" t="n">
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Bauer et al. 2013</t>
+        </is>
+      </c>
+      <c r="G27" t="n">
         <v>2013</v>
       </c>
-      <c r="G27" t="n">
+      <c r="H27" t="n">
+        <v>750</v>
+      </c>
+      <c r="I27" t="n">
         <v>2788013.925</v>
       </c>
-      <c r="H27" t="n">
+      <c r="J27" t="n">
+        <v>3994531.496985722</v>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>Amine scrubbing</t>
+        </is>
+      </c>
+      <c r="L27" t="n">
         <v>3994531.496985722</v>
       </c>
     </row>
@@ -1312,13 +1748,29 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F28" t="n">
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Bauer et al. 2013</t>
+        </is>
+      </c>
+      <c r="G28" t="n">
         <v>2013</v>
       </c>
-      <c r="G28" t="n">
+      <c r="H28" t="n">
+        <v>1000</v>
+      </c>
+      <c r="I28" t="n">
         <v>3186111.9</v>
       </c>
-      <c r="H28" t="n">
+      <c r="J28" t="n">
+        <v>4564907.019777896</v>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>Amine scrubbing</t>
+        </is>
+      </c>
+      <c r="L28" t="n">
         <v>4564907.019777896</v>
       </c>
     </row>
@@ -1344,13 +1796,29 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F29" t="n">
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Bauer et al. 2013</t>
+        </is>
+      </c>
+      <c r="G29" t="n">
         <v>2013</v>
       </c>
-      <c r="G29" t="n">
+      <c r="H29" t="n">
+        <v>1250</v>
+      </c>
+      <c r="I29" t="n">
         <v>3539386.5</v>
       </c>
-      <c r="H29" t="n">
+      <c r="J29" t="n">
+        <v>5071061.778952935</v>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>Amine scrubbing</t>
+        </is>
+      </c>
+      <c r="L29" t="n">
         <v>5071061.778952935</v>
       </c>
     </row>
@@ -1376,13 +1844,29 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F30" t="n">
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Bauer et al. 2013</t>
+        </is>
+      </c>
+      <c r="G30" t="n">
         <v>2013</v>
       </c>
-      <c r="G30" t="n">
+      <c r="H30" t="n">
+        <v>1500</v>
+      </c>
+      <c r="I30" t="n">
         <v>3759187.05</v>
       </c>
-      <c r="H30" t="n">
+      <c r="J30" t="n">
+        <v>5385981.375356955</v>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>Amine scrubbing</t>
+        </is>
+      </c>
+      <c r="L30" t="n">
         <v>5385981.375356955</v>
       </c>
     </row>
@@ -1408,13 +1892,29 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F31" t="n">
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Bauer et al. 2013</t>
+        </is>
+      </c>
+      <c r="G31" t="n">
         <v>2013</v>
       </c>
-      <c r="G31" t="n">
+      <c r="H31" t="n">
+        <v>1750</v>
+      </c>
+      <c r="I31" t="n">
         <v>3804674.475</v>
       </c>
-      <c r="H31" t="n">
+      <c r="J31" t="n">
+        <v>5451153.557694342</v>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>Amine scrubbing</t>
+        </is>
+      </c>
+      <c r="L31" t="n">
         <v>5451153.557694342</v>
       </c>
     </row>
@@ -1440,13 +1940,29 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F32" t="n">
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Bauer et al. 2013</t>
+        </is>
+      </c>
+      <c r="G32" t="n">
         <v>2013</v>
       </c>
-      <c r="G32" t="n">
+      <c r="H32" t="n">
+        <v>1800</v>
+      </c>
+      <c r="I32" t="n">
         <v>3810584.52</v>
       </c>
-      <c r="H32" t="n">
+      <c r="J32" t="n">
+        <v>5459621.184304601</v>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>Amine scrubbing</t>
+        </is>
+      </c>
+      <c r="L32" t="n">
         <v>5459621.184304601</v>
       </c>
     </row>
@@ -1472,13 +1988,29 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F33" t="n">
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Bauer et al. 2013</t>
+        </is>
+      </c>
+      <c r="G33" t="n">
         <v>2013</v>
       </c>
-      <c r="G33" t="n">
+      <c r="H33" t="n">
+        <v>250</v>
+      </c>
+      <c r="I33" t="n">
         <v>1454269.5</v>
       </c>
-      <c r="H33" t="n">
+      <c r="J33" t="n">
+        <v>2083606.997355896</v>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>Physical absorption (organic solvent)</t>
+        </is>
+      </c>
+      <c r="L33" t="n">
         <v>2083606.997355896</v>
       </c>
     </row>
@@ -1504,13 +2036,29 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F34" t="n">
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Bauer et al. 2013</t>
+        </is>
+      </c>
+      <c r="G34" t="n">
         <v>2013</v>
       </c>
-      <c r="G34" t="n">
+      <c r="H34" t="n">
+        <v>500</v>
+      </c>
+      <c r="I34" t="n">
         <v>2182732.35</v>
       </c>
-      <c r="H34" t="n">
+      <c r="J34" t="n">
+        <v>3127313.333474352</v>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>Physical absorption (organic solvent)</t>
+        </is>
+      </c>
+      <c r="L34" t="n">
         <v>3127313.333474352</v>
       </c>
     </row>
@@ -1536,13 +2084,29 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F35" t="n">
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Bauer et al. 2013</t>
+        </is>
+      </c>
+      <c r="G35" t="n">
         <v>2013</v>
       </c>
-      <c r="G35" t="n">
+      <c r="H35" t="n">
+        <v>750</v>
+      </c>
+      <c r="I35" t="n">
         <v>2562900.975</v>
       </c>
-      <c r="H35" t="n">
+      <c r="J35" t="n">
+        <v>3672000.550819672</v>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>Physical absorption (organic solvent)</t>
+        </is>
+      </c>
+      <c r="L35" t="n">
         <v>3672000.550819672</v>
       </c>
     </row>
@@ -1568,13 +2132,29 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F36" t="n">
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Bauer et al. 2013</t>
+        </is>
+      </c>
+      <c r="G36" t="n">
         <v>2013</v>
       </c>
-      <c r="G36" t="n">
+      <c r="H36" t="n">
+        <v>1000</v>
+      </c>
+      <c r="I36" t="n">
         <v>2806275.3</v>
       </c>
-      <c r="H36" t="n">
+      <c r="J36" t="n">
+        <v>4020695.511792703</v>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>Physical absorption (organic solvent)</t>
+        </is>
+      </c>
+      <c r="L36" t="n">
         <v>4020695.511792703</v>
       </c>
     </row>
@@ -1600,13 +2180,29 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F37" t="n">
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Bauer et al. 2013</t>
+        </is>
+      </c>
+      <c r="G37" t="n">
         <v>2013</v>
       </c>
-      <c r="G37" t="n">
+      <c r="H37" t="n">
+        <v>1250</v>
+      </c>
+      <c r="I37" t="n">
         <v>3016447.125</v>
       </c>
-      <c r="H37" t="n">
+      <c r="J37" t="n">
+        <v>4321819.536753041</v>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>Physical absorption (organic solvent)</t>
+        </is>
+      </c>
+      <c r="L37" t="n">
         <v>4321819.536753041</v>
       </c>
     </row>
@@ -1632,13 +2228,29 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F38" t="n">
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Bauer et al. 2013</t>
+        </is>
+      </c>
+      <c r="G38" t="n">
         <v>2013</v>
       </c>
-      <c r="G38" t="n">
+      <c r="H38" t="n">
+        <v>1500</v>
+      </c>
+      <c r="I38" t="n">
         <v>3233259.45</v>
       </c>
-      <c r="H38" t="n">
+      <c r="J38" t="n">
+        <v>4632457.748915917</v>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>Physical absorption (organic solvent)</t>
+        </is>
+      </c>
+      <c r="L38" t="n">
         <v>4632457.748915917</v>
       </c>
     </row>
@@ -1664,13 +2276,29 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F39" t="n">
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Bauer et al. 2013</t>
+        </is>
+      </c>
+      <c r="G39" t="n">
         <v>2013</v>
       </c>
-      <c r="G39" t="n">
+      <c r="H39" t="n">
+        <v>1750</v>
+      </c>
+      <c r="I39" t="n">
         <v>3479289.975</v>
       </c>
-      <c r="H39" t="n">
+      <c r="J39" t="n">
+        <v>4984958.384769963</v>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>Physical absorption (organic solvent)</t>
+        </is>
+      </c>
+      <c r="L39" t="n">
         <v>4984958.384769963</v>
       </c>
     </row>
@@ -1696,13 +2324,29 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F40" t="n">
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Bauer et al. 2013</t>
+        </is>
+      </c>
+      <c r="G40" t="n">
         <v>2013</v>
       </c>
-      <c r="G40" t="n">
+      <c r="H40" t="n">
+        <v>2000</v>
+      </c>
+      <c r="I40" t="n">
         <v>3859458.6</v>
       </c>
-      <c r="H40" t="n">
+      <c r="J40" t="n">
+        <v>5529645.602115283</v>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>Physical absorption (organic solvent)</t>
+        </is>
+      </c>
+      <c r="L40" t="n">
         <v>5529645.602115283</v>
       </c>
     </row>
@@ -1728,13 +2372,29 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F41" t="n">
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Bauer et al. 2013</t>
+        </is>
+      </c>
+      <c r="G41" t="n">
         <v>2013</v>
       </c>
-      <c r="G41" t="n">
+      <c r="H41" t="n">
+        <v>500</v>
+      </c>
+      <c r="I41" t="n">
         <v>1460910</v>
       </c>
-      <c r="H41" t="n">
+      <c r="J41" t="n">
+        <v>2093121.184558435</v>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>Pressure swing adsorption</t>
+        </is>
+      </c>
+      <c r="L41" t="n">
         <v>2093121.184558435</v>
       </c>
     </row>
@@ -1760,13 +2420,29 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F42" t="n">
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Bauer et al. 2013</t>
+        </is>
+      </c>
+      <c r="G42" t="n">
         <v>2013</v>
       </c>
-      <c r="G42" t="n">
+      <c r="H42" t="n">
+        <v>500</v>
+      </c>
+      <c r="I42" t="n">
         <v>1859340</v>
       </c>
-      <c r="H42" t="n">
+      <c r="J42" t="n">
+        <v>2663972.416710735</v>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>Pressure swing adsorption</t>
+        </is>
+      </c>
+      <c r="L42" t="n">
         <v>2663972.416710735</v>
       </c>
     </row>
@@ -1792,13 +2468,29 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F43" t="n">
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Bauer et al. 2013</t>
+        </is>
+      </c>
+      <c r="G43" t="n">
         <v>2013</v>
       </c>
-      <c r="G43" t="n">
+      <c r="H43" t="n">
+        <v>60</v>
+      </c>
+      <c r="I43" t="n">
         <v>504678</v>
       </c>
-      <c r="H43" t="n">
+      <c r="J43" t="n">
+        <v>723078.2273929138</v>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>Water scrubbing</t>
+        </is>
+      </c>
+      <c r="L43" t="n">
         <v>723078.2273929138</v>
       </c>
     </row>
@@ -1824,13 +2516,29 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F44" t="n">
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Bauer et al. 2013</t>
+        </is>
+      </c>
+      <c r="G44" t="n">
         <v>2013</v>
       </c>
-      <c r="G44" t="n">
+      <c r="H44" t="n">
+        <v>72</v>
+      </c>
+      <c r="I44" t="n">
         <v>478116</v>
       </c>
-      <c r="H44" t="n">
+      <c r="J44" t="n">
+        <v>685021.4785827604</v>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>Water scrubbing</t>
+        </is>
+      </c>
+      <c r="L44" t="n">
         <v>685021.4785827604</v>
       </c>
     </row>
@@ -1856,20 +2564,36 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F45" t="n">
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Bauer et al. 2013</t>
+        </is>
+      </c>
+      <c r="G45" t="n">
         <v>2013</v>
       </c>
-      <c r="G45" t="n">
+      <c r="H45" t="n">
+        <v>72</v>
+      </c>
+      <c r="I45" t="n">
         <v>610926</v>
       </c>
-      <c r="H45" t="n">
+      <c r="J45" t="n">
+        <v>875305.2226335272</v>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>Water scrubbing</t>
+        </is>
+      </c>
+      <c r="L45" t="n">
         <v>875305.2226335272</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t xml:space="preserve">Membrane separation </t>
+          <t>Membrane separation</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -1888,20 +2612,30 @@
           <t>m3_per_hr</t>
         </is>
       </c>
-      <c r="F46" t="n">
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Hagen et al. 2001</t>
+        </is>
+      </c>
+      <c r="G46" t="n">
         <v>2001</v>
       </c>
-      <c r="G46" t="n">
+      <c r="H46" t="n">
+        <v>298</v>
+      </c>
+      <c r="I46" t="n">
         <v>29891545.6</v>
       </c>
-      <c r="H46" t="n">
+      <c r="J46" t="n">
         <v>61617672.49221404</v>
       </c>
+      <c r="K46" t="inlineStr"/>
+      <c r="L46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t xml:space="preserve">Membrane separation </t>
+          <t>Membrane separation</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -1920,20 +2654,30 @@
           <t>m3_per_hr</t>
         </is>
       </c>
-      <c r="F47" t="n">
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Hagen et al. 2001</t>
+        </is>
+      </c>
+      <c r="G47" t="n">
         <v>2001</v>
       </c>
-      <c r="G47" t="n">
+      <c r="H47" t="n">
+        <v>373</v>
+      </c>
+      <c r="I47" t="n">
         <v>23317304.24</v>
       </c>
-      <c r="H47" t="n">
+      <c r="J47" t="n">
         <v>48065698.41813847</v>
       </c>
+      <c r="K47" t="inlineStr"/>
+      <c r="L47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t xml:space="preserve">Membrane separation </t>
+          <t>Membrane separation</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -1952,20 +2696,30 @@
           <t>m3_per_hr</t>
         </is>
       </c>
-      <c r="F48" t="n">
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Hagen et al. 2001</t>
+        </is>
+      </c>
+      <c r="G48" t="n">
         <v>2001</v>
       </c>
-      <c r="G48" t="n">
+      <c r="H48" t="n">
+        <v>398</v>
+      </c>
+      <c r="I48" t="n">
         <v>31260559.76</v>
       </c>
-      <c r="H48" t="n">
+      <c r="J48" t="n">
         <v>64439723.49208216</v>
       </c>
+      <c r="K48" t="inlineStr"/>
+      <c r="L48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t xml:space="preserve">Membrane separation </t>
+          <t>Membrane separation</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -1984,20 +2738,30 @@
           <t>m3_per_hr</t>
         </is>
       </c>
-      <c r="F49" t="n">
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Hagen et al. 2001</t>
+        </is>
+      </c>
+      <c r="G49" t="n">
         <v>2001</v>
       </c>
-      <c r="G49" t="n">
+      <c r="H49" t="n">
+        <v>622</v>
+      </c>
+      <c r="I49" t="n">
         <v>24009423.92</v>
       </c>
-      <c r="H49" t="n">
+      <c r="J49" t="n">
         <v>49492416.3382602</v>
       </c>
+      <c r="K49" t="inlineStr"/>
+      <c r="L49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t xml:space="preserve">Membrane separation </t>
+          <t>Membrane separation</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -2016,20 +2780,30 @@
           <t>m3_per_hr</t>
         </is>
       </c>
-      <c r="F50" t="n">
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Hagen et al. 2001</t>
+        </is>
+      </c>
+      <c r="G50" t="n">
         <v>2001</v>
       </c>
-      <c r="G50" t="n">
+      <c r="H50" t="n">
+        <v>997</v>
+      </c>
+      <c r="I50" t="n">
         <v>71433056</v>
       </c>
-      <c r="H50" t="n">
+      <c r="J50" t="n">
         <v>147250286.3728126</v>
       </c>
+      <c r="K50" t="inlineStr"/>
+      <c r="L50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t xml:space="preserve">Membrane separation </t>
+          <t>Membrane separation</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2048,15 +2822,25 @@
           <t>m3_per_hr</t>
         </is>
       </c>
-      <c r="F51" t="n">
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Hagen et al. 2001</t>
+        </is>
+      </c>
+      <c r="G51" t="n">
         <v>2001</v>
       </c>
-      <c r="G51" t="n">
+      <c r="H51" t="n">
+        <v>1597</v>
+      </c>
+      <c r="I51" t="n">
         <v>81096490.44</v>
       </c>
-      <c r="H51" t="n">
+      <c r="J51" t="n">
         <v>167170244.5590464</v>
       </c>
+      <c r="K51" t="inlineStr"/>
+      <c r="L51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -2080,13 +2864,29 @@
           <t>m3_per_hr</t>
         </is>
       </c>
-      <c r="F52" t="n">
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Hagen et al. 2001</t>
+        </is>
+      </c>
+      <c r="G52" t="n">
         <v>2001</v>
       </c>
-      <c r="G52" t="n">
+      <c r="H52" t="n">
+        <v>800</v>
+      </c>
+      <c r="I52" t="n">
         <v>1110544</v>
       </c>
-      <c r="H52" t="n">
+      <c r="J52" t="n">
+        <v>2289247.180319554</v>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>Pressure swing adsorption</t>
+        </is>
+      </c>
+      <c r="L52" t="n">
         <v>2289247.180319554</v>
       </c>
     </row>
@@ -2112,13 +2912,29 @@
           <t>m3_per_hr</t>
         </is>
       </c>
-      <c r="F53" t="n">
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Hagen et al. 2001</t>
+        </is>
+      </c>
+      <c r="G53" t="n">
         <v>2001</v>
       </c>
-      <c r="G53" t="n">
+      <c r="H53" t="n">
+        <v>200</v>
+      </c>
+      <c r="I53" t="n">
         <v>770216</v>
       </c>
-      <c r="H53" t="n">
+      <c r="J53" t="n">
+        <v>1587703.689576464</v>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>Water scrubbing</t>
+        </is>
+      </c>
+      <c r="L53" t="n">
         <v>1587703.689576464</v>
       </c>
     </row>
@@ -2144,20 +2960,36 @@
           <t>m3_per_hr</t>
         </is>
       </c>
-      <c r="F54" t="n">
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>Hagen et al. 2001</t>
+        </is>
+      </c>
+      <c r="G54" t="n">
         <v>2001</v>
       </c>
-      <c r="G54" t="n">
+      <c r="H54" t="n">
+        <v>660</v>
+      </c>
+      <c r="I54" t="n">
         <v>2239000</v>
       </c>
-      <c r="H54" t="n">
+      <c r="J54" t="n">
+        <v>4615417.702257165</v>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>Water scrubbing</t>
+        </is>
+      </c>
+      <c r="L54" t="n">
         <v>4615417.702257165</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t xml:space="preserve">Membrane separation </t>
+          <t>Membrane separation</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -2176,20 +3008,30 @@
           <t>m3_per_hr</t>
         </is>
       </c>
-      <c r="F55" t="n">
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Hagen et al. 2001</t>
+        </is>
+      </c>
+      <c r="G55" t="n">
         <v>2001</v>
       </c>
-      <c r="G55" t="n">
+      <c r="H55" t="n">
+        <v>400</v>
+      </c>
+      <c r="I55" t="n">
         <v>34928.4</v>
       </c>
-      <c r="H55" t="n">
+      <c r="J55" t="n">
         <v>72000.51615521176</v>
       </c>
+      <c r="K55" t="inlineStr"/>
+      <c r="L55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t xml:space="preserve">Membrane separation </t>
+          <t>Membrane separation</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -2208,15 +3050,25 @@
           <t>m3_per_hr</t>
         </is>
       </c>
-      <c r="F56" t="n">
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>Hagen et al. 2001</t>
+        </is>
+      </c>
+      <c r="G56" t="n">
         <v>2001</v>
       </c>
-      <c r="G56" t="n">
+      <c r="H56" t="n">
+        <v>1600</v>
+      </c>
+      <c r="I56" t="n">
         <v>72543.59999999999</v>
       </c>
-      <c r="H56" t="n">
+      <c r="J56" t="n">
         <v>149539.5335531321</v>
       </c>
+      <c r="K56" t="inlineStr"/>
+      <c r="L56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -2240,15 +3092,25 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F57" t="n">
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>Persson et al. 2006</t>
+        </is>
+      </c>
+      <c r="G57" t="n">
         <v>2006</v>
       </c>
-      <c r="G57" t="n">
+      <c r="H57" t="n">
+        <v>300</v>
+      </c>
+      <c r="I57" t="n">
         <v>1255600</v>
       </c>
-      <c r="H57" t="n">
+      <c r="J57" t="n">
         <v>2042737.550040032</v>
       </c>
+      <c r="K57" t="inlineStr"/>
+      <c r="L57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -2272,15 +3134,25 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F58" t="n">
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>Allegue &amp; Hinge 2012</t>
+        </is>
+      </c>
+      <c r="G58" t="n">
         <v>2012</v>
       </c>
-      <c r="G58" t="n">
+      <c r="H58" t="n">
+        <v>500</v>
+      </c>
+      <c r="I58" t="n">
         <v>1284800</v>
       </c>
-      <c r="H58" t="n">
+      <c r="J58" t="n">
         <v>1786324.734861444</v>
       </c>
+      <c r="K58" t="inlineStr"/>
+      <c r="L58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -2304,13 +3176,29 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F59" t="n">
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>Urban et al. 2008 (Fraunhofer UMSICHT)</t>
+        </is>
+      </c>
+      <c r="G59" t="n">
         <v>2008</v>
       </c>
-      <c r="G59" t="n">
+      <c r="H59" t="n">
+        <v>250</v>
+      </c>
+      <c r="I59" t="n">
         <v>1684066</v>
       </c>
-      <c r="H59" t="n">
+      <c r="J59" t="n">
+        <v>2378882.246784846</v>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>Water scrubbing</t>
+        </is>
+      </c>
+      <c r="L59" t="n">
         <v>2378882.246784846</v>
       </c>
     </row>
@@ -2336,13 +3224,29 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F60" t="n">
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>Urban et al. 2008 (Fraunhofer UMSICHT)</t>
+        </is>
+      </c>
+      <c r="G60" t="n">
         <v>2008</v>
       </c>
-      <c r="G60" t="n">
+      <c r="H60" t="n">
+        <v>500</v>
+      </c>
+      <c r="I60" t="n">
         <v>1946603.8</v>
       </c>
-      <c r="H60" t="n">
+      <c r="J60" t="n">
+        <v>2749738.562113313</v>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>Water scrubbing</t>
+        </is>
+      </c>
+      <c r="L60" t="n">
         <v>2749738.562113313</v>
       </c>
     </row>
@@ -2368,13 +3272,29 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F61" t="n">
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>Urban et al. 2008 (Fraunhofer UMSICHT)</t>
+        </is>
+      </c>
+      <c r="G61" t="n">
         <v>2008</v>
       </c>
-      <c r="G61" t="n">
+      <c r="H61" t="n">
+        <v>1000</v>
+      </c>
+      <c r="I61" t="n">
         <v>2498889.2</v>
       </c>
-      <c r="H61" t="n">
+      <c r="J61" t="n">
+        <v>3529887.281473758</v>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>Water scrubbing</t>
+        </is>
+      </c>
+      <c r="L61" t="n">
         <v>3529887.281473758</v>
       </c>
     </row>
@@ -2400,13 +3320,29 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F62" t="n">
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>Urban et al. 2008 (Fraunhofer UMSICHT)</t>
+        </is>
+      </c>
+      <c r="G62" t="n">
         <v>2008</v>
       </c>
-      <c r="G62" t="n">
+      <c r="H62" t="n">
+        <v>500</v>
+      </c>
+      <c r="I62" t="n">
         <v>2070151</v>
       </c>
-      <c r="H62" t="n">
+      <c r="J62" t="n">
+        <v>2924259.181091415</v>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>Pressure swing adsorption</t>
+        </is>
+      </c>
+      <c r="L62" t="n">
         <v>2924259.181091415</v>
       </c>
     </row>
@@ -2432,13 +3368,29 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F63" t="n">
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>Urban et al. 2008 (Fraunhofer UMSICHT)</t>
+        </is>
+      </c>
+      <c r="G63" t="n">
         <v>2008</v>
       </c>
-      <c r="G63" t="n">
+      <c r="H63" t="n">
+        <v>1000</v>
+      </c>
+      <c r="I63" t="n">
         <v>2707448.64</v>
       </c>
-      <c r="H63" t="n">
+      <c r="J63" t="n">
+        <v>3824494.707320125</v>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>Pressure swing adsorption</t>
+        </is>
+      </c>
+      <c r="L63" t="n">
         <v>3824494.707320125</v>
       </c>
     </row>
@@ -2464,13 +3416,29 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F64" t="n">
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>Urban et al. 2008 (Fraunhofer UMSICHT)</t>
+        </is>
+      </c>
+      <c r="G64" t="n">
         <v>2008</v>
       </c>
-      <c r="G64" t="n">
+      <c r="H64" t="n">
+        <v>2000</v>
+      </c>
+      <c r="I64" t="n">
         <v>4302090</v>
       </c>
-      <c r="H64" t="n">
+      <c r="J64" t="n">
+        <v>6077057.267987487</v>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>Pressure swing adsorption</t>
+        </is>
+      </c>
+      <c r="L64" t="n">
         <v>6077057.267987487</v>
       </c>
     </row>
@@ -2496,13 +3464,29 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F65" t="n">
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>Urban et al. 2008 (Fraunhofer UMSICHT)</t>
+        </is>
+      </c>
+      <c r="G65" t="n">
         <v>2008</v>
       </c>
-      <c r="G65" t="n">
+      <c r="H65" t="n">
+        <v>500</v>
+      </c>
+      <c r="I65" t="n">
         <v>1465210.96</v>
       </c>
-      <c r="H65" t="n">
+      <c r="J65" t="n">
+        <v>2069731.436023636</v>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>Amine scrubbing</t>
+        </is>
+      </c>
+      <c r="L65" t="n">
         <v>2069731.436023636</v>
       </c>
     </row>
@@ -2528,13 +3512,29 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F66" t="n">
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>Urban et al. 2008 (Fraunhofer UMSICHT)</t>
+        </is>
+      </c>
+      <c r="G66" t="n">
         <v>2008</v>
       </c>
-      <c r="G66" t="n">
+      <c r="H66" t="n">
+        <v>500</v>
+      </c>
+      <c r="I66" t="n">
         <v>1571696.88</v>
       </c>
-      <c r="H66" t="n">
+      <c r="J66" t="n">
+        <v>2220151.588571429</v>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>Pressure swing adsorption</t>
+        </is>
+      </c>
+      <c r="L66" t="n">
         <v>2220151.588571429</v>
       </c>
     </row>
@@ -2560,13 +3560,29 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F67" t="n">
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>Urban et al. 2008 (Fraunhofer UMSICHT)</t>
+        </is>
+      </c>
+      <c r="G67" t="n">
         <v>2008</v>
       </c>
-      <c r="G67" t="n">
+      <c r="H67" t="n">
+        <v>250</v>
+      </c>
+      <c r="I67" t="n">
         <v>1246355.92</v>
       </c>
-      <c r="H67" t="n">
+      <c r="J67" t="n">
+        <v>1760580.625262426</v>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>Amine scrubbing</t>
+        </is>
+      </c>
+      <c r="L67" t="n">
         <v>1760580.625262426</v>
       </c>
     </row>
@@ -2592,13 +3608,29 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F68" t="n">
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>Urban et al. 2008 (Fraunhofer UMSICHT)</t>
+        </is>
+      </c>
+      <c r="G68" t="n">
         <v>2008</v>
       </c>
-      <c r="G68" t="n">
+      <c r="H68" t="n">
+        <v>500</v>
+      </c>
+      <c r="I68" t="n">
         <v>1555223.92</v>
       </c>
-      <c r="H68" t="n">
+      <c r="J68" t="n">
+        <v>2196882.172707682</v>
+      </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>Amine scrubbing</t>
+        </is>
+      </c>
+      <c r="L68" t="n">
         <v>2196882.172707682</v>
       </c>
     </row>
@@ -2624,13 +3656,29 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F69" t="n">
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>Urban et al. 2008 (Fraunhofer UMSICHT)</t>
+        </is>
+      </c>
+      <c r="G69" t="n">
         <v>2008</v>
       </c>
-      <c r="G69" t="n">
+      <c r="H69" t="n">
+        <v>1000</v>
+      </c>
+      <c r="I69" t="n">
         <v>2288711.88</v>
       </c>
-      <c r="H69" t="n">
+      <c r="J69" t="n">
+        <v>3232994.466569344</v>
+      </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>Amine scrubbing</t>
+        </is>
+      </c>
+      <c r="L69" t="n">
         <v>3232994.466569344</v>
       </c>
     </row>
@@ -2656,13 +3704,29 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F70" t="n">
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>Electrigaz Technologies Inc.2011</t>
+        </is>
+      </c>
+      <c r="G70" t="n">
         <v>2011</v>
       </c>
-      <c r="G70" t="n">
+      <c r="H70" t="n">
+        <v>127</v>
+      </c>
+      <c r="I70" t="n">
         <v>1977000</v>
       </c>
-      <c r="H70" t="n">
+      <c r="J70" t="n">
+        <v>2743564.28205566</v>
+      </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>Water scrubbing</t>
+        </is>
+      </c>
+      <c r="L70" t="n">
         <v>2743564.28205566</v>
       </c>
     </row>
@@ -2688,13 +3752,29 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F71" t="n">
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>Electrigaz Technologies Inc.2011</t>
+        </is>
+      </c>
+      <c r="G71" t="n">
         <v>2011</v>
       </c>
-      <c r="G71" t="n">
+      <c r="H71" t="n">
+        <v>300</v>
+      </c>
+      <c r="I71" t="n">
         <v>2030000</v>
       </c>
-      <c r="H71" t="n">
+      <c r="J71" t="n">
+        <v>2817114.563769848</v>
+      </c>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>Water scrubbing</t>
+        </is>
+      </c>
+      <c r="L71" t="n">
         <v>2817114.563769848</v>
       </c>
     </row>
@@ -2720,13 +3800,29 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F72" t="n">
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>Electrigaz Technologies Inc.2011</t>
+        </is>
+      </c>
+      <c r="G72" t="n">
         <v>2011</v>
       </c>
-      <c r="G72" t="n">
+      <c r="H72" t="n">
+        <v>450</v>
+      </c>
+      <c r="I72" t="n">
         <v>2896000</v>
       </c>
-      <c r="H72" t="n">
+      <c r="J72" t="n">
+        <v>4018898.412156393</v>
+      </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>Water scrubbing</t>
+        </is>
+      </c>
+      <c r="L72" t="n">
         <v>4018898.412156393</v>
       </c>
     </row>
@@ -2752,13 +3848,29 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F73" t="n">
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>Electrigaz Technologies Inc.2011</t>
+        </is>
+      </c>
+      <c r="G73" t="n">
         <v>2011</v>
       </c>
-      <c r="G73" t="n">
+      <c r="H73" t="n">
+        <v>700</v>
+      </c>
+      <c r="I73" t="n">
         <v>3713000</v>
       </c>
-      <c r="H73" t="n">
+      <c r="J73" t="n">
+        <v>5152682.943486426</v>
+      </c>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>Water scrubbing</t>
+        </is>
+      </c>
+      <c r="L73" t="n">
         <v>5152682.943486426</v>
       </c>
     </row>
@@ -2784,20 +3896,36 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F74" t="n">
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>Electrigaz Technologies Inc.2011</t>
+        </is>
+      </c>
+      <c r="G74" t="n">
         <v>2011</v>
       </c>
-      <c r="G74" t="n">
+      <c r="H74" t="n">
+        <v>900</v>
+      </c>
+      <c r="I74" t="n">
         <v>4163000</v>
       </c>
-      <c r="H74" t="n">
+      <c r="J74" t="n">
+        <v>5777166.467474815</v>
+      </c>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>Water scrubbing</t>
+        </is>
+      </c>
+      <c r="L74" t="n">
         <v>5777166.467474815</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Water scrubbing</t>
+          <t>Water scrubbing + PSA (O2/N2 removal)</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -2816,20 +3944,36 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F75" t="n">
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>Electrigaz Technologies Inc.2011</t>
+        </is>
+      </c>
+      <c r="G75" t="n">
         <v>2011</v>
       </c>
-      <c r="G75" t="n">
+      <c r="H75" t="n">
+        <v>475</v>
+      </c>
+      <c r="I75" t="n">
         <v>4405000</v>
       </c>
-      <c r="H75" t="n">
+      <c r="J75" t="n">
+        <v>6112999.829264128</v>
+      </c>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>Water scrubbing + PSA (O2/N2 removal)</t>
+        </is>
+      </c>
+      <c r="L75" t="n">
         <v>6112999.829264128</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Water scrubbing</t>
+          <t>Water scrubbing + PSA (O2/N2 removal)</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -2848,13 +3992,29 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F76" t="n">
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>Electrigaz Technologies Inc.2011</t>
+        </is>
+      </c>
+      <c r="G76" t="n">
         <v>2011</v>
       </c>
-      <c r="G76" t="n">
+      <c r="H76" t="n">
+        <v>1110</v>
+      </c>
+      <c r="I76" t="n">
         <v>6773000</v>
       </c>
-      <c r="H76" t="n">
+      <c r="J76" t="n">
+        <v>9399170.906607477</v>
+      </c>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>Water scrubbing + PSA (O2/N2 removal)</t>
+        </is>
+      </c>
+      <c r="L76" t="n">
         <v>9399170.906607477</v>
       </c>
     </row>
@@ -2880,15 +4040,25 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F77" t="n">
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>Electrigaz Technologies Inc.2011</t>
+        </is>
+      </c>
+      <c r="G77" t="n">
         <v>2011</v>
       </c>
-      <c r="G77" t="n">
+      <c r="H77" t="n">
+        <v>3960</v>
+      </c>
+      <c r="I77" t="n">
         <v>10263000</v>
       </c>
-      <c r="H77" t="n">
+      <c r="J77" t="n">
         <v>14242387.57042854</v>
       </c>
+      <c r="K77" t="inlineStr"/>
+      <c r="L77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -2912,13 +4082,29 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F78" t="n">
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>Muñoz et al. 2015</t>
+        </is>
+      </c>
+      <c r="G78" t="n">
         <v>2015</v>
       </c>
-      <c r="G78" t="n">
+      <c r="H78" t="n">
+        <v>100</v>
+      </c>
+      <c r="I78" t="n">
         <v>610225</v>
       </c>
-      <c r="H78" t="n">
+      <c r="J78" t="n">
+        <v>890788.2183908047</v>
+      </c>
+      <c r="K78" t="inlineStr">
+        <is>
+          <t>Water scrubbing</t>
+        </is>
+      </c>
+      <c r="L78" t="n">
         <v>890788.2183908047</v>
       </c>
     </row>
@@ -2944,13 +4130,29 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F79" t="n">
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>Muñoz et al. 2015</t>
+        </is>
+      </c>
+      <c r="G79" t="n">
         <v>2015</v>
       </c>
-      <c r="G79" t="n">
+      <c r="H79" t="n">
+        <v>500</v>
+      </c>
+      <c r="I79" t="n">
         <v>1386875</v>
       </c>
-      <c r="H79" t="n">
+      <c r="J79" t="n">
+        <v>2024518.67816092</v>
+      </c>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t>Water scrubbing</t>
+        </is>
+      </c>
+      <c r="L79" t="n">
         <v>2024518.67816092</v>
       </c>
     </row>
@@ -2976,13 +4178,29 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F80" t="n">
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>Muñoz et al. 2015</t>
+        </is>
+      </c>
+      <c r="G80" t="n">
         <v>2015</v>
       </c>
-      <c r="G80" t="n">
+      <c r="H80" t="n">
+        <v>1000</v>
+      </c>
+      <c r="I80" t="n">
         <v>1997100</v>
       </c>
-      <c r="H80" t="n">
+      <c r="J80" t="n">
+        <v>2915306.896551724</v>
+      </c>
+      <c r="K80" t="inlineStr">
+        <is>
+          <t>Water scrubbing</t>
+        </is>
+      </c>
+      <c r="L80" t="n">
         <v>2915306.896551724</v>
       </c>
     </row>
@@ -3008,13 +4226,29 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F81" t="n">
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>Muñoz et al. 2015</t>
+        </is>
+      </c>
+      <c r="G81" t="n">
         <v>2015</v>
       </c>
-      <c r="G81" t="n">
+      <c r="H81" t="n">
+        <v>1000</v>
+      </c>
+      <c r="I81" t="n">
         <v>2219000</v>
       </c>
-      <c r="H81" t="n">
+      <c r="J81" t="n">
+        <v>3239229.885057472</v>
+      </c>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t>Water scrubbing</t>
+        </is>
+      </c>
+      <c r="L81" t="n">
         <v>3239229.885057472</v>
       </c>
     </row>
@@ -3040,13 +4274,29 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F82" t="n">
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>Muñoz et al. 2015</t>
+        </is>
+      </c>
+      <c r="G82" t="n">
         <v>2015</v>
       </c>
-      <c r="G82" t="n">
+      <c r="H82" t="n">
+        <v>250</v>
+      </c>
+      <c r="I82" t="n">
         <v>1248187.5</v>
       </c>
-      <c r="H82" t="n">
+      <c r="J82" t="n">
+        <v>1822066.810344828</v>
+      </c>
+      <c r="K82" t="inlineStr">
+        <is>
+          <t>Physical absorption (organic solvent)</t>
+        </is>
+      </c>
+      <c r="L82" t="n">
         <v>1822066.810344828</v>
       </c>
     </row>
@@ -3072,13 +4322,29 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F83" t="n">
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>Muñoz et al. 2015</t>
+        </is>
+      </c>
+      <c r="G83" t="n">
         <v>2015</v>
       </c>
-      <c r="G83" t="n">
+      <c r="H83" t="n">
+        <v>1000</v>
+      </c>
+      <c r="I83" t="n">
         <v>2219000</v>
       </c>
-      <c r="H83" t="n">
+      <c r="J83" t="n">
+        <v>3239229.885057472</v>
+      </c>
+      <c r="K83" t="inlineStr">
+        <is>
+          <t>Physical absorption (organic solvent)</t>
+        </is>
+      </c>
+      <c r="L83" t="n">
         <v>3239229.885057472</v>
       </c>
     </row>
@@ -3104,13 +4370,29 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F84" t="n">
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>Muñoz et al. 2015</t>
+        </is>
+      </c>
+      <c r="G84" t="n">
         <v>2015</v>
       </c>
-      <c r="G84" t="n">
+      <c r="H84" t="n">
+        <v>1500</v>
+      </c>
+      <c r="I84" t="n">
         <v>2496375</v>
       </c>
-      <c r="H84" t="n">
+      <c r="J84" t="n">
+        <v>3644133.620689656</v>
+      </c>
+      <c r="K84" t="inlineStr">
+        <is>
+          <t>Physical absorption (organic solvent)</t>
+        </is>
+      </c>
+      <c r="L84" t="n">
         <v>3644133.620689656</v>
       </c>
     </row>
@@ -3136,13 +4418,29 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F85" t="n">
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>Muñoz et al. 2015</t>
+        </is>
+      </c>
+      <c r="G85" t="n">
         <v>2015</v>
       </c>
-      <c r="G85" t="n">
+      <c r="H85" t="n">
+        <v>600</v>
+      </c>
+      <c r="I85" t="n">
         <v>2130240</v>
       </c>
-      <c r="H85" t="n">
+      <c r="J85" t="n">
+        <v>3109660.689655173</v>
+      </c>
+      <c r="K85" t="inlineStr">
+        <is>
+          <t>Amine scrubbing</t>
+        </is>
+      </c>
+      <c r="L85" t="n">
         <v>3109660.689655173</v>
       </c>
     </row>
@@ -3168,13 +4466,29 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F86" t="n">
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>Muñoz et al. 2015</t>
+        </is>
+      </c>
+      <c r="G86" t="n">
         <v>2015</v>
       </c>
-      <c r="G86" t="n">
+      <c r="H86" t="n">
+        <v>1800</v>
+      </c>
+      <c r="I86" t="n">
         <v>2995650</v>
       </c>
-      <c r="H86" t="n">
+      <c r="J86" t="n">
+        <v>4372960.344827587</v>
+      </c>
+      <c r="K86" t="inlineStr">
+        <is>
+          <t>Amine scrubbing</t>
+        </is>
+      </c>
+      <c r="L86" t="n">
         <v>4372960.344827587</v>
       </c>
     </row>
@@ -3200,13 +4514,29 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F87" t="n">
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>Muñoz et al. 2015</t>
+        </is>
+      </c>
+      <c r="G87" t="n">
         <v>2015</v>
       </c>
-      <c r="G87" t="n">
+      <c r="H87" t="n">
+        <v>600</v>
+      </c>
+      <c r="I87" t="n">
         <v>1797390</v>
       </c>
-      <c r="H87" t="n">
+      <c r="J87" t="n">
+        <v>2623776.206896552</v>
+      </c>
+      <c r="K87" t="inlineStr">
+        <is>
+          <t>Pressure swing adsorption</t>
+        </is>
+      </c>
+      <c r="L87" t="n">
         <v>2623776.206896552</v>
       </c>
     </row>
@@ -3232,20 +4562,36 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F88" t="n">
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>Muñoz et al. 2015</t>
+        </is>
+      </c>
+      <c r="G88" t="n">
         <v>2015</v>
       </c>
-      <c r="G88" t="n">
+      <c r="H88" t="n">
+        <v>2000</v>
+      </c>
+      <c r="I88" t="n">
         <v>3328500</v>
       </c>
-      <c r="H88" t="n">
+      <c r="J88" t="n">
+        <v>4858844.827586208</v>
+      </c>
+      <c r="K88" t="inlineStr">
+        <is>
+          <t>Pressure swing adsorption</t>
+        </is>
+      </c>
+      <c r="L88" t="n">
         <v>4858844.827586208</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t xml:space="preserve">Membrane separation </t>
+          <t>Membrane separation</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -3264,20 +4610,36 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F89" t="n">
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>Muñoz et al. 2015</t>
+        </is>
+      </c>
+      <c r="G89" t="n">
         <v>2015</v>
       </c>
-      <c r="G89" t="n">
+      <c r="H89" t="n">
+        <v>100</v>
+      </c>
+      <c r="I89" t="n">
         <v>665700</v>
       </c>
-      <c r="H89" t="n">
+      <c r="J89" t="n">
+        <v>971768.9655172414</v>
+      </c>
+      <c r="K89" t="inlineStr">
+        <is>
+          <t>Membrane separation</t>
+        </is>
+      </c>
+      <c r="L89" t="n">
         <v>971768.9655172414</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t xml:space="preserve">Membrane separation </t>
+          <t>Membrane separation</t>
         </is>
       </c>
       <c r="B90" t="n">
@@ -3296,20 +4658,36 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F90" t="n">
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>Muñoz et al. 2015</t>
+        </is>
+      </c>
+      <c r="G90" t="n">
         <v>2015</v>
       </c>
-      <c r="G90" t="n">
+      <c r="H90" t="n">
+        <v>400</v>
+      </c>
+      <c r="I90" t="n">
         <v>1109500</v>
       </c>
-      <c r="H90" t="n">
+      <c r="J90" t="n">
+        <v>1619614.942528736</v>
+      </c>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t>Membrane separation</t>
+        </is>
+      </c>
+      <c r="L90" t="n">
         <v>1619614.942528736</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t xml:space="preserve">Membrane separation </t>
+          <t>Membrane separation</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -3328,13 +4706,29 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F91" t="n">
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>Muñoz et al. 2015</t>
+        </is>
+      </c>
+      <c r="G91" t="n">
         <v>2015</v>
       </c>
-      <c r="G91" t="n">
+      <c r="H91" t="n">
+        <v>1000</v>
+      </c>
+      <c r="I91" t="n">
         <v>2219000</v>
       </c>
-      <c r="H91" t="n">
+      <c r="J91" t="n">
+        <v>3239229.885057472</v>
+      </c>
+      <c r="K91" t="inlineStr">
+        <is>
+          <t>Membrane separation</t>
+        </is>
+      </c>
+      <c r="L91" t="n">
         <v>3239229.885057472</v>
       </c>
     </row>
@@ -3360,13 +4754,29 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F92" t="n">
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>Kapoor et al. 2019</t>
+        </is>
+      </c>
+      <c r="G92" t="n">
         <v>2019</v>
       </c>
-      <c r="G92" t="n">
+      <c r="H92" t="n">
+        <v>100</v>
+      </c>
+      <c r="I92" t="n">
         <v>615725</v>
       </c>
-      <c r="H92" t="n">
+      <c r="J92" t="n">
+        <v>823804.5761316872</v>
+      </c>
+      <c r="K92" t="inlineStr">
+        <is>
+          <t>Water scrubbing</t>
+        </is>
+      </c>
+      <c r="L92" t="n">
         <v>823804.5761316872</v>
       </c>
     </row>
@@ -3392,13 +4802,29 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F93" t="n">
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>Kapoor et al. 2019</t>
+        </is>
+      </c>
+      <c r="G93" t="n">
         <v>2019</v>
       </c>
-      <c r="G93" t="n">
+      <c r="H93" t="n">
+        <v>500</v>
+      </c>
+      <c r="I93" t="n">
         <v>1399375</v>
       </c>
-      <c r="H93" t="n">
+      <c r="J93" t="n">
+        <v>1872283.127572016</v>
+      </c>
+      <c r="K93" t="inlineStr">
+        <is>
+          <t>Water scrubbing</t>
+        </is>
+      </c>
+      <c r="L93" t="n">
         <v>1872283.127572016</v>
       </c>
     </row>
@@ -3424,13 +4850,29 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F94" t="n">
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>Kapoor et al. 2019</t>
+        </is>
+      </c>
+      <c r="G94" t="n">
         <v>2019</v>
       </c>
-      <c r="G94" t="n">
+      <c r="H94" t="n">
+        <v>1000</v>
+      </c>
+      <c r="I94" t="n">
         <v>2015100</v>
       </c>
-      <c r="H94" t="n">
+      <c r="J94" t="n">
+        <v>2696087.703703703</v>
+      </c>
+      <c r="K94" t="inlineStr">
+        <is>
+          <t>Water scrubbing</t>
+        </is>
+      </c>
+      <c r="L94" t="n">
         <v>2696087.703703703</v>
       </c>
     </row>
@@ -3456,13 +4898,29 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F95" t="n">
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>Kapoor et al. 2019</t>
+        </is>
+      </c>
+      <c r="G95" t="n">
         <v>2019</v>
       </c>
-      <c r="G95" t="n">
+      <c r="H95" t="n">
+        <v>1000</v>
+      </c>
+      <c r="I95" t="n">
         <v>2239000</v>
       </c>
-      <c r="H95" t="n">
+      <c r="J95" t="n">
+        <v>2995653.004115226</v>
+      </c>
+      <c r="K95" t="inlineStr">
+        <is>
+          <t>Water scrubbing</t>
+        </is>
+      </c>
+      <c r="L95" t="n">
         <v>2995653.004115226</v>
       </c>
     </row>
@@ -3488,13 +4946,29 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F96" t="n">
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>Kapoor et al. 2019</t>
+        </is>
+      </c>
+      <c r="G96" t="n">
         <v>2019</v>
       </c>
-      <c r="G96" t="n">
+      <c r="H96" t="n">
+        <v>250</v>
+      </c>
+      <c r="I96" t="n">
         <v>1259437.5</v>
       </c>
-      <c r="H96" t="n">
+      <c r="J96" t="n">
+        <v>1685054.814814815</v>
+      </c>
+      <c r="K96" t="inlineStr">
+        <is>
+          <t>Physical absorption (organic solvent)</t>
+        </is>
+      </c>
+      <c r="L96" t="n">
         <v>1685054.814814815</v>
       </c>
     </row>
@@ -3520,13 +4994,29 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F97" t="n">
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>Kapoor et al. 2019</t>
+        </is>
+      </c>
+      <c r="G97" t="n">
         <v>2019</v>
       </c>
-      <c r="G97" t="n">
+      <c r="H97" t="n">
+        <v>1000</v>
+      </c>
+      <c r="I97" t="n">
         <v>2239000</v>
       </c>
-      <c r="H97" t="n">
+      <c r="J97" t="n">
+        <v>2995653.004115226</v>
+      </c>
+      <c r="K97" t="inlineStr">
+        <is>
+          <t>Physical absorption (organic solvent)</t>
+        </is>
+      </c>
+      <c r="L97" t="n">
         <v>2995653.004115226</v>
       </c>
     </row>
@@ -3552,13 +5042,29 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F98" t="n">
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>Kapoor et al. 2019</t>
+        </is>
+      </c>
+      <c r="G98" t="n">
         <v>2019</v>
       </c>
-      <c r="G98" t="n">
+      <c r="H98" t="n">
+        <v>1500</v>
+      </c>
+      <c r="I98" t="n">
         <v>2518875</v>
       </c>
-      <c r="H98" t="n">
+      <c r="J98" t="n">
+        <v>3370109.62962963</v>
+      </c>
+      <c r="K98" t="inlineStr">
+        <is>
+          <t>Physical absorption (organic solvent)</t>
+        </is>
+      </c>
+      <c r="L98" t="n">
         <v>3370109.62962963</v>
       </c>
     </row>
@@ -3584,13 +5090,29 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F99" t="n">
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>Kapoor et al. 2019</t>
+        </is>
+      </c>
+      <c r="G99" t="n">
         <v>2019</v>
       </c>
-      <c r="G99" t="n">
+      <c r="H99" t="n">
+        <v>600</v>
+      </c>
+      <c r="I99" t="n">
         <v>2149440</v>
       </c>
-      <c r="H99" t="n">
+      <c r="J99" t="n">
+        <v>2875826.883950617</v>
+      </c>
+      <c r="K99" t="inlineStr">
+        <is>
+          <t>Amine scrubbing</t>
+        </is>
+      </c>
+      <c r="L99" t="n">
         <v>2875826.883950617</v>
       </c>
     </row>
@@ -3616,13 +5138,29 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F100" t="n">
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>Kapoor et al. 2019</t>
+        </is>
+      </c>
+      <c r="G100" t="n">
         <v>2019</v>
       </c>
-      <c r="G100" t="n">
+      <c r="H100" t="n">
+        <v>1800</v>
+      </c>
+      <c r="I100" t="n">
         <v>3022650</v>
       </c>
-      <c r="H100" t="n">
+      <c r="J100" t="n">
+        <v>4044131.555555556</v>
+      </c>
+      <c r="K100" t="inlineStr">
+        <is>
+          <t>Amine scrubbing</t>
+        </is>
+      </c>
+      <c r="L100" t="n">
         <v>4044131.555555556</v>
       </c>
     </row>
@@ -3648,13 +5186,29 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F101" t="n">
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>Kapoor et al. 2019</t>
+        </is>
+      </c>
+      <c r="G101" t="n">
         <v>2019</v>
       </c>
-      <c r="G101" t="n">
+      <c r="H101" t="n">
+        <v>600</v>
+      </c>
+      <c r="I101" t="n">
         <v>1813590</v>
       </c>
-      <c r="H101" t="n">
+      <c r="J101" t="n">
+        <v>2426478.933333333</v>
+      </c>
+      <c r="K101" t="inlineStr">
+        <is>
+          <t>Pressure swing adsorption</t>
+        </is>
+      </c>
+      <c r="L101" t="n">
         <v>2426478.933333333</v>
       </c>
     </row>
@@ -3680,20 +5234,36 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F102" t="n">
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>Kapoor et al. 2019</t>
+        </is>
+      </c>
+      <c r="G102" t="n">
         <v>2019</v>
       </c>
-      <c r="G102" t="n">
+      <c r="H102" t="n">
+        <v>2000</v>
+      </c>
+      <c r="I102" t="n">
         <v>3358500</v>
       </c>
-      <c r="H102" t="n">
+      <c r="J102" t="n">
+        <v>4493479.50617284</v>
+      </c>
+      <c r="K102" t="inlineStr">
+        <is>
+          <t>Pressure swing adsorption</t>
+        </is>
+      </c>
+      <c r="L102" t="n">
         <v>4493479.50617284</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t xml:space="preserve">Membrane separation </t>
+          <t>Membrane separation</t>
         </is>
       </c>
       <c r="B103" t="n">
@@ -3712,20 +5282,36 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F103" t="n">
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>Kapoor et al. 2019</t>
+        </is>
+      </c>
+      <c r="G103" t="n">
         <v>2019</v>
       </c>
-      <c r="G103" t="n">
+      <c r="H103" t="n">
+        <v>100</v>
+      </c>
+      <c r="I103" t="n">
         <v>279875</v>
       </c>
-      <c r="H103" t="n">
+      <c r="J103" t="n">
+        <v>374456.6255144033</v>
+      </c>
+      <c r="K103" t="inlineStr">
+        <is>
+          <t>Membrane separation</t>
+        </is>
+      </c>
+      <c r="L103" t="n">
         <v>374456.6255144033</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t xml:space="preserve">Membrane separation </t>
+          <t>Membrane separation</t>
         </is>
       </c>
       <c r="B104" t="n">
@@ -3744,20 +5330,36 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F104" t="n">
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>Kapoor et al. 2019</t>
+        </is>
+      </c>
+      <c r="G104" t="n">
         <v>2019</v>
       </c>
-      <c r="G104" t="n">
+      <c r="H104" t="n">
+        <v>400</v>
+      </c>
+      <c r="I104" t="n">
         <v>2686800</v>
       </c>
-      <c r="H104" t="n">
+      <c r="J104" t="n">
+        <v>3594783.604938271</v>
+      </c>
+      <c r="K104" t="inlineStr">
+        <is>
+          <t>Membrane separation</t>
+        </is>
+      </c>
+      <c r="L104" t="n">
         <v>3594783.604938271</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t xml:space="preserve">Membrane separation </t>
+          <t>Membrane separation</t>
         </is>
       </c>
       <c r="B105" t="n">
@@ -3776,20 +5378,36 @@
           <t>nm3_per_hr</t>
         </is>
       </c>
-      <c r="F105" t="n">
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>Kapoor et al. 2019</t>
+        </is>
+      </c>
+      <c r="G105" t="n">
         <v>2019</v>
       </c>
-      <c r="G105" t="n">
+      <c r="H105" t="n">
+        <v>1000</v>
+      </c>
+      <c r="I105" t="n">
         <v>2239000</v>
       </c>
-      <c r="H105" t="n">
+      <c r="J105" t="n">
+        <v>2995653.004115226</v>
+      </c>
+      <c r="K105" t="inlineStr">
+        <is>
+          <t>Membrane separation</t>
+        </is>
+      </c>
+      <c r="L105" t="n">
         <v>2995653.004115226</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Siloxane removal system</t>
+          <t>Siloxane removal system, siloxane-only (ancillary, not upgrading)</t>
         </is>
       </c>
       <c r="B106" t="n">
@@ -3801,22 +5419,32 @@
         </is>
       </c>
       <c r="D106" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>scfm</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>South Coast AQMD toolkit manual 2014</t>
+        </is>
+      </c>
+      <c r="G106" t="n">
+        <v>2014</v>
+      </c>
+      <c r="H106" t="n">
         <v>1699</v>
       </c>
-      <c r="E106" t="inlineStr">
-        <is>
-          <t>m3_per_hr</t>
-        </is>
-      </c>
-      <c r="F106" t="n">
-        <v>2014</v>
-      </c>
-      <c r="G106" t="n">
+      <c r="I106" t="n">
         <v>1163849</v>
       </c>
-      <c r="H106" t="n">
+      <c r="J106" t="n">
         <v>1642035.180003471</v>
       </c>
+      <c r="K106" t="inlineStr"/>
+      <c r="L106" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>